<commit_message>
feat(desktop,backend,frontend): implement quota flexible breaks, 1-1 penalties, client robustness fixes, visual timelines, and custom branding icon
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F46"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1329,9 +1329,49 @@
         <v>* [COMPLETED] TSK-ATT-026 (Filter live-status activity logs query to the current date): Resolved a bug where employees who haven't sent desktop events today were showing old offline-synced sleep/lock times from previous days (e.g. June 26th) in their live status metadata and being incorrectly marked as AWAY. Refactored the GET /api/attendance/live-status endpoint in routes.ts to filter desktopActivityLogs selection to only include events occurring greater than or equal to the start of today.</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="B45" s="2" t="str">
+        <v>TSK-ATT-027</v>
+      </c>
+      <c r="C45" s="2" t="str">
+        <v>Align desktop agent activity log and break naming logic with web dashboard</v>
+      </c>
+      <c r="D45" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E45" s="2" t="str">
+        <v>Resolved a misalignment between the desktop agent console activity log and the web dashboard workday timeline event log. Refactored DashboardForm.cs to utilize a GetScheduledBreakInfo helper mapping lock/idle break states to specific scheduled name strings (Morning Tea Break, Lunch Break, Evening Tea Break) only when they fall inside configured break hours or were manually started. Filtered out redundant logs and transient breaks under 1 minute from the desktop list box view.</v>
+      </c>
+      <c r="F45" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-027 (Align desktop agent activity log and break naming logic with web dashboard): Resolved a misalignment between the desktop agent console activity log and the web dashboard workday timeline event log. Refactored DashboardForm.cs to utilize a GetScheduledBreakInfo helper mapping lock/idle break states to specific scheduled name strings (Morning Tea Break, Lunch Break, Evening Tea Break) only when they fall inside configured break hours or were manually started. Filtered out redundant logs and transient breaks under 1 minute from the desktop list box view.</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="B46" s="2" t="str">
+        <v>TSK-ATT-028</v>
+      </c>
+      <c r="C46" s="2" t="str">
+        <v>Implement Quota-Based Flexible Breaks, Penalties &amp; Desktop Agent Robustness</v>
+      </c>
+      <c r="D46" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E46" s="2" t="str">
+        <v>Refactored the Express backend /break/end API and visual workday timeline components to support wide flexible scheduled break windows (tea and lunch windows spanning up to 3 hours), 10m/20m minimum duration limits, and first-qualifying-break quota check per window. Implemented critical C# desktop client robustness fixes: added CancellationTokens for 30s timeouts to prevent UI freezes on checkout, quoted Application.ExecutablePath in the startup registry key, introduced a 3-attempt data refresh retry loop, used local machine-level DPAPI password storage for silent auto-login, forced tray status updates to refresh the hidden dashboard state, filtered out idle logs &lt; 10 minutes from Event Logs and visual bars, resolved high-DPI layout clipping and maximized control spacing by expanding action widths to 48%, increasing label sizing heights, centering button layout panels dynamically when maximized, and added support for loading custom application branding icon dynamically from the executable's resources.</v>
+      </c>
+      <c r="F46" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-028 (Implement Quota-Based Flexible Breaks, Penalties &amp; Desktop Agent Robustness): Refactored the Express backend /break/end API and visual workday timeline components to support wide flexible scheduled break windows (tea and lunch windows spanning up to 3 hours), 10m/20m minimum duration limits, and first-qualifying-break quota check per window. Implemented critical C# desktop client robustness fixes: added CancellationTokens for 30s timeouts to prevent UI freezes on checkout, quoted Application.ExecutablePath in the startup registry key, introduced a 3-attempt data refresh retry loop, used local machine-level DPAPI password storage for silent auto-login, forced tray status updates to refresh the hidden dashboard state, filtered out idle logs &lt; 10 minutes from Event Logs and visual bars, resolved high-DPI layout clipping and maximized control spacing by expanding action widths to 48%, increasing label sizing heights, centering button layout panels dynamically when maximized, and added support for loading custom application branding icon dynamically from the executable's resources.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F46"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2263,7 +2303,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W64"/>
+  <dimension ref="A1:W66"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -6834,9 +6874,151 @@
         <v>Completed bug fixes and dashboard features: (1) Added token guard to WorkdayTimeline.tsx. (2) Eliminated hero section white flash on .dashboard-hero. (3) Added dynamic relatable thoughts pools. (4) Redesigned hero layouts. (5) Fixed the desktop offline sync date mapping logic. (6) Filtered out duplicate/redundant timeline log items. (7) Classified locks/idle times as breaks only during scheduled hours. (8) Aligned desktop reminder triggers. (9) Published and packaged the self-contained Release build. (10) Added a current-date filter to /live-status desktop logs check to prevent stale historical events from showing up as active status details.</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="B65" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C65" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D65" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E65" s="2" t="str">
+        <v>Desktop Client App</v>
+      </c>
+      <c r="F65" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G65" s="2" t="str">
+        <v>Desktop Event Log Formatting</v>
+      </c>
+      <c r="H65" s="2" t="str">
+        <v>TSK-ATT-027</v>
+      </c>
+      <c r="I65" s="2" t="str">
+        <v>Align desktop agent activity log and break naming logic with web dashboard</v>
+      </c>
+      <c r="J65" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K65" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L65" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M65" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N65" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O65" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P65" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q65" s="2">
+        <v>4</v>
+      </c>
+      <c r="R65" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S65" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T65" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U65" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="V65" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="W65" s="2" t="str">
+        <v>Aligned desktop log console formatting with web dashboard. Refactored /break/end backend route and workday timeline visuals to support wide flexible break ranges, duration thresholds, and direct 1-to-1 penalty calculations. Implemented 6 critical C# desktop client fixes: resolved UI freezing via checkout timeout, quoted startup registry path, added startup fetch retries, enabled secure DPAPI password persistence for silent re-login, enforced dashboard polls while hidden, filtered out idle logs &lt; 10 minutes, resolved high-DPI layout clipping, and added dynamic custom branding icon support.</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="B66" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C66" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D66" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E66" s="2" t="str">
+        <v>Desktop Client / Web Dashboard</v>
+      </c>
+      <c r="F66" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G66" s="2" t="str">
+        <v>Flexible Breaks, Penalties &amp; Agent Robustness</v>
+      </c>
+      <c r="H66" s="2" t="str">
+        <v>TSK-ATT-028</v>
+      </c>
+      <c r="I66" s="2" t="str">
+        <v>Implement Quota-Based Flexible Breaks, Penalties &amp; Desktop Agent Robustness</v>
+      </c>
+      <c r="J66" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K66" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L66" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M66" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="N66" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O66" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P66" s="2">
+        <v>6</v>
+      </c>
+      <c r="Q66" s="2">
+        <v>4</v>
+      </c>
+      <c r="R66" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S66" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T66" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U66" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="V66" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="W66" s="2" t="str">
+        <v>Aligned desktop log console formatting with web dashboard. Refactored /break/end backend route and workday timeline visuals to support wide flexible break ranges, duration thresholds, and direct 1-to-1 penalty calculations. Implemented 6 critical C# desktop client fixes: resolved UI freezing via checkout timeout, quoted startup registry path, added startup fetch retries, enabled secure DPAPI password persistence for silent re-login, enforced dashboard polls while hidden, filtered out idle logs &lt; 10 minutes, resolved high-DPI layout clipping, and added dynamic custom branding icon support.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W66"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: workday timeline bounding guard and desktop agent self-healing
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F48"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1369,9 +1369,49 @@
         <v>* [COMPLETED] TSK-ATT-028 (Implement Quota-Based Flexible Breaks, Penalties &amp; Desktop Agent Robustness): Refactored the Express backend /break/end API and visual workday timeline components to support wide flexible scheduled break windows (tea and lunch windows spanning up to 3 hours), 10m/20m minimum duration limits, and first-qualifying-break quota check per window. Implemented critical C# desktop client robustness fixes: added CancellationTokens for 30s timeouts to prevent UI freezes on checkout, quoted Application.ExecutablePath in the startup registry key, introduced a 3-attempt data refresh retry loop, used local machine-level DPAPI password storage for silent auto-login, forced tray status updates to refresh the hidden dashboard state, filtered out idle logs &lt; 10 minutes from Event Logs and visual bars, resolved high-DPI layout clipping and maximized control spacing by expanding action widths to 48%, increasing label sizing heights, centering button layout panels dynamically when maximized, and added support for loading custom application branding icon dynamically from the executable's resources.</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="B47" s="2" t="str">
+        <v>TSK-ATT-029</v>
+      </c>
+      <c r="C47" s="2" t="str">
+        <v>Deduplicate consecutive identical events in workday timeline</v>
+      </c>
+      <c r="D47" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E47" s="2" t="str">
+        <v>Implemented a consecutive identical event filter inside the WorkdayTimeline.tsx React component's combined log logic to deduplicate contiguous matching desktop events (such as multiple 'Screen Locked' alerts) occurring within 60 seconds of each other.</v>
+      </c>
+      <c r="F47" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-029 (Deduplicate consecutive identical events in workday timeline): Implemented a consecutive identical event filter inside the WorkdayTimeline.tsx React component's combined log logic to deduplicate contiguous matching desktop events (such as multiple 'Screen Locked' alerts) occurring within 60 seconds of each other.</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="B48" s="2" t="str">
+        <v>TSK-ATT-030</v>
+      </c>
+      <c r="C48" s="2" t="str">
+        <v>Filter out pre-checkin events and restore manual checkin active status on live-status</v>
+      </c>
+      <c r="D48" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E48" s="2" t="str">
+        <v>Updated the GET /api/attendance/live-status endpoint in routes.ts to filter and ignore desktop activity logs recorded prior to the employee's check-in timestamp, and removed the offline agent check from the status mapper to ensure manually checked-in users display as ACTIVE rather than OFFLINE.</v>
+      </c>
+      <c r="F48" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-030 (Filter out pre-checkin events and restore manual checkin active status on live-status): Updated the GET /api/attendance/live-status endpoint in routes.ts to filter and ignore desktop activity logs recorded prior to the employee's check-in timestamp, and removed the offline agent check from the status mapper to ensure manually checked-in users display as ACTIVE rather than OFFLINE.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F48"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2303,7 +2343,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W66"/>
+  <dimension ref="A1:W68"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -6924,7 +6964,7 @@
         <v>1</v>
       </c>
       <c r="Q65" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R65" s="2" t="str">
         <v>100%</v>
@@ -6995,7 +7035,7 @@
         <v>6</v>
       </c>
       <c r="Q66" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R66" s="2" t="str">
         <v>100%</v>
@@ -7016,9 +7056,151 @@
         <v>Aligned desktop log console formatting with web dashboard. Refactored /break/end backend route and workday timeline visuals to support wide flexible break ranges, duration thresholds, and direct 1-to-1 penalty calculations. Implemented 6 critical C# desktop client fixes: resolved UI freezing via checkout timeout, quoted startup registry path, added startup fetch retries, enabled secure DPAPI password persistence for silent re-login, enforced dashboard polls while hidden, filtered out idle logs &lt; 10 minutes, resolved high-DPI layout clipping, and added dynamic custom branding icon support.</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="B67" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C67" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D67" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E67" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F67" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G67" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H67" s="2" t="str">
+        <v>TSK-ATT-029</v>
+      </c>
+      <c r="I67" s="2" t="str">
+        <v>Work on task</v>
+      </c>
+      <c r="J67" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K67" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L67" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M67" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N67" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="O67" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P67" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q67" s="2">
+        <v>2</v>
+      </c>
+      <c r="R67" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S67" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T67" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U67" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="V67" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="W67" s="2" t="str">
+        <v>Aligned desktop log console formatting with web dashboard. Refactored /break/end backend route and workday timeline visuals to support wide flexible break ranges, duration thresholds, and direct 1-to-1 penalty calculations. Implemented 6 critical C# desktop client fixes: resolved UI freezing via checkout timeout, quoted startup registry path, added startup fetch retries, enabled secure DPAPI password persistence for silent re-login, enforced dashboard polls while hidden, filtered out idle logs &lt; 10 minutes, resolved high-DPI layout clipping, and added dynamic custom branding icon support.</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="B68" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C68" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D68" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E68" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F68" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G68" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H68" s="2" t="str">
+        <v>TSK-ATT-030</v>
+      </c>
+      <c r="I68" s="2" t="str">
+        <v>Work on task</v>
+      </c>
+      <c r="J68" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K68" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L68" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M68" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N68" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="O68" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P68" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q68" s="2">
+        <v>2</v>
+      </c>
+      <c r="R68" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S68" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T68" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U68" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="V68" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="W68" s="2" t="str">
+        <v>Aligned desktop log console formatting with web dashboard. Refactored /break/end backend route and workday timeline visuals to support wide flexible break ranges, duration thresholds, and direct 1-to-1 penalty calculations. Implemented 6 critical C# desktop client fixes: resolved UI freezing via checkout timeout, quoted startup registry path, added startup fetch retries, enabled secure DPAPI password persistence for silent re-login, enforced dashboard polls while hidden, filtered out idle logs &lt; 10 minutes, resolved high-DPI layout clipping, and added dynamic custom branding icon support.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W68"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(dashboard): resolve hero section white strip rendering bug and sync project sheets
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F50"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1409,9 +1409,49 @@
         <v>* [COMPLETED] TSK-ATT-030 (Filter out pre-checkin events and restore manual checkin active status on live-status): Updated the GET /api/attendance/live-status endpoint in routes.ts to filter and ignore desktop activity logs recorded prior to the employee's check-in timestamp, and removed the offline agent check from the status mapper to ensure manually checked-in users display as ACTIVE rather than OFFLINE.</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="2" t="str">
+        <v>2026-07-03</v>
+      </c>
+      <c r="B49" s="2" t="str">
+        <v>TSK-ATT-029</v>
+      </c>
+      <c r="C49" s="2" t="str">
+        <v>Implement Offline Attendance Export &amp; Resolve Google Sheets Sync Queue Blockers</v>
+      </c>
+      <c r="D49" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E49" s="2" t="str">
+        <v>Resolved Google Sheets API 'caller does not have permission' errors for July 2026 spreadsheet creation by implementing diagnostic and queue reset utilities (check-google-sheets-db.ts and reset-failed-syncs.ts). Extended the Google Sheets backfiller range to July 31st. Created a backend GET /api/attendance/export route that compiles all active employee attendance logs for a chosen month/year into a styled spreadsheet. Added month selection controls and a 'Download Report' button to the HR/Admin web panel header to trigger browser-side downloads. Completely disabled the background Google Sheets sync queueing and processing loop in code using a DISABLE_GOOGLE_SHEETS_SYNC environment flag in .env, and configured docker-compose.prod.yml to forward this flag to the production container.</v>
+      </c>
+      <c r="F49" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-029 (Implement Offline Attendance Export &amp; Resolve Google Sheets Sync Queue Blockers): Resolved Google Sheets API 'caller does not have permission' errors for July 2026 spreadsheet creation by implementing diagnostic and queue reset utilities (check-google-sheets-db.ts and reset-failed-syncs.ts). Extended the Google Sheets backfiller range to July 31st. Created a backend GET /api/attendance/export route that compiles all active employee attendance logs for a chosen month/year into a styled spreadsheet. Added month selection controls and a 'Download Report' button to the HR/Admin web panel header to trigger browser-side downloads. Completely disabled the background Google Sheets sync queueing and processing loop in code using a DISABLE_GOOGLE_SHEETS_SYNC environment flag in .env, and configured docker-compose.prod.yml to forward this flag to the production container.</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="str">
+        <v>2026-07-06</v>
+      </c>
+      <c r="B50" s="2" t="str">
+        <v>TSK-ATT-031</v>
+      </c>
+      <c r="C50" s="2" t="str">
+        <v>Resolve Dashboard Hero Section White Strip Bug</v>
+      </c>
+      <c r="D50" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E50" s="2" t="str">
+        <v>Resolved a layout rendering bug where a mysterious horizontal white strip appeared across the middle of the dashboard's hero section card. The card base styling (.card) applied a semi-transparent white background and backdrop-filter, which bled through when individual background properties were overridden. Fixed this by applying a clean background shorthand with !important and setting backdrop-filter to none.</v>
+      </c>
+      <c r="F50" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-031 (Resolve Dashboard Hero Section White Strip Bug): Resolved a layout rendering bug where a mysterious horizontal white strip appeared across the middle of the dashboard's hero section card. The card base styling (.card) applied a semi-transparent white background and backdrop-filter, which bled through when individual background properties were overridden. Fixed this by applying a clean background shorthand with !important and setting backdrop-filter to none.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F50"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2343,7 +2383,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W68"/>
+  <dimension ref="A1:W70"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -7070,40 +7110,40 @@
         <v>Sprint 4</v>
       </c>
       <c r="E67" s="2" t="str">
-        <v>N/A</v>
+        <v>HR Panel / Attendance Page</v>
       </c>
       <c r="F67" s="2" t="str">
-        <v>N/A</v>
+        <v>Attendance</v>
       </c>
       <c r="G67" s="2" t="str">
-        <v>N/A</v>
+        <v>Offline Export &amp; Google Sheets Sync</v>
       </c>
       <c r="H67" s="2" t="str">
         <v>TSK-ATT-029</v>
       </c>
       <c r="I67" s="2" t="str">
-        <v>Work on task</v>
+        <v>Implement Offline Attendance Export &amp; Resolve Google Sheets Sync Queue Blockers</v>
       </c>
       <c r="J67" s="2" t="str">
-        <v>N/A</v>
+        <v>COMPLETED</v>
       </c>
       <c r="K67" s="2" t="str">
-        <v>N/A</v>
+        <v>COMPLETED</v>
       </c>
       <c r="L67" s="2" t="str">
         <v>N/A</v>
       </c>
       <c r="M67" s="2" t="str">
-        <v>N/A</v>
+        <v>COMPLETED</v>
       </c>
       <c r="N67" s="2" t="str">
-        <v>N/A</v>
+        <v>COMPLETED</v>
       </c>
       <c r="O67" s="2" t="str">
-        <v>MEDIUM</v>
+        <v>HIGH</v>
       </c>
       <c r="P67" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q67" s="2">
         <v>2</v>
@@ -7118,10 +7158,10 @@
         <v>None</v>
       </c>
       <c r="U67" s="2" t="str">
-        <v>2026-07-02</v>
+        <v>2026-07-03</v>
       </c>
       <c r="V67" s="2" t="str">
-        <v>2026-07-02</v>
+        <v>2026-07-03</v>
       </c>
       <c r="W67" s="2" t="str">
         <v>Aligned desktop log console formatting with web dashboard. Refactored /break/end backend route and workday timeline visuals to support wide flexible break ranges, duration thresholds, and direct 1-to-1 penalty calculations. Implemented 6 critical C# desktop client fixes: resolved UI freezing via checkout timeout, quoted startup registry path, added startup fetch retries, enabled secure DPAPI password persistence for silent re-login, enforced dashboard polls while hidden, filtered out idle logs &lt; 10 minutes, resolved high-DPI layout clipping, and added dynamic custom branding icon support.</v>
@@ -7198,9 +7238,151 @@
         <v>Aligned desktop log console formatting with web dashboard. Refactored /break/end backend route and workday timeline visuals to support wide flexible break ranges, duration thresholds, and direct 1-to-1 penalty calculations. Implemented 6 critical C# desktop client fixes: resolved UI freezing via checkout timeout, quoted startup registry path, added startup fetch retries, enabled secure DPAPI password persistence for silent re-login, enforced dashboard polls while hidden, filtered out idle logs &lt; 10 minutes, resolved high-DPI layout clipping, and added dynamic custom branding icon support.</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="2" t="str">
+        <v>2026-07-03</v>
+      </c>
+      <c r="B69" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C69" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D69" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E69" s="2" t="str">
+        <v>HR Panel / Attendance Page</v>
+      </c>
+      <c r="F69" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G69" s="2" t="str">
+        <v>Offline Export &amp; Google Sheets Sync</v>
+      </c>
+      <c r="H69" s="2" t="str">
+        <v>TSK-ATT-029</v>
+      </c>
+      <c r="I69" s="2" t="str">
+        <v>Implement Offline Attendance Export &amp; Resolve Google Sheets Sync Queue Blockers</v>
+      </c>
+      <c r="J69" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K69" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L69" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M69" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="N69" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O69" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P69" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q69" s="2">
+        <v>4</v>
+      </c>
+      <c r="R69" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S69" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T69" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U69" s="2" t="str">
+        <v>2026-07-03</v>
+      </c>
+      <c r="V69" s="2" t="str">
+        <v>2026-07-03</v>
+      </c>
+      <c r="W69" s="2" t="str">
+        <v>Created database diagnostic and queue reset utilities to manage failed Google Sheets sync tasks. Extended backfill range up to July 31. Implemented styled monthly offline Excel attendance sheet export in the Express backend, and added interactive download controls to the frontend HR panel. Disabled background Google Sheets queueing and worker sync loops via .env flag, and updated the Docker compose configuration to pass the environment setting to production.</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="str">
+        <v>2026-07-06</v>
+      </c>
+      <c r="B70" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C70" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D70" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E70" s="2" t="str">
+        <v>Dashboard Page</v>
+      </c>
+      <c r="F70" s="2" t="str">
+        <v>Dashboard UI</v>
+      </c>
+      <c r="G70" s="2" t="str">
+        <v>Hero Section Layout Fix</v>
+      </c>
+      <c r="H70" s="2" t="str">
+        <v>TSK-ATT-031</v>
+      </c>
+      <c r="I70" s="2" t="str">
+        <v>Resolve Dashboard Hero Section White Strip Bug</v>
+      </c>
+      <c r="J70" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K70" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L70" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M70" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N70" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O70" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P70" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q70" s="2">
+        <v>1</v>
+      </c>
+      <c r="R70" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S70" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T70" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U70" s="2" t="str">
+        <v>2026-07-06</v>
+      </c>
+      <c r="V70" s="2" t="str">
+        <v>2026-07-06</v>
+      </c>
+      <c r="W70" s="2" t="str">
+        <v>Successfully resolved the dashboard hero section layout rendering bug by completely overriding the .card background shorthand and disabling backdrop-filters on .dashboard-hero.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W70"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(desktop): implement resilient silent reconnect on startup and sync sheet
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1449,9 +1449,29 @@
         <v>* [COMPLETED] TSK-ATT-031 (Resolve Dashboard Hero Section White Strip Bug): Resolved a layout rendering bug where a mysterious horizontal white strip appeared across the middle of the dashboard's hero section card. The card base styling (.card) applied a semi-transparent white background and backdrop-filter, which bled through when individual background properties were overridden. Fixed this by applying a clean background shorthand with !important and setting backdrop-filter to none.</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="2" t="str">
+        <v>2026-07-06</v>
+      </c>
+      <c r="B51" s="2" t="str">
+        <v>TSK-ATT-032</v>
+      </c>
+      <c r="C51" s="2" t="str">
+        <v>Implement resilient silent re-authentication on system startup</v>
+      </c>
+      <c r="D51" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E51" s="2" t="str">
+        <v>Resolved a startup auto-login bug in the C# desktop agent application. During boot-time launch, slow local network interface connection speeds caused initial silent token refreshes to fail with network exceptions, prompting the login credentials dialog immediately. Introduced a transient network error flag to run silently in system tray during offline startup, and configured background timers and network change address listeners to trigger silent re-authentication once connection is restored.</v>
+      </c>
+      <c r="F51" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-032 (Implement resilient silent re-authentication on system startup): Resolved a startup auto-login bug in the C# desktop agent application. During boot-time launch, slow local network interface connection speeds caused initial silent token refreshes to fail with network exceptions, prompting the login credentials dialog immediately. Introduced a transient network error flag to run silently in system tray during offline startup, and configured background timers and network change address listeners to trigger silent re-authentication once connection is restored.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F51"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2383,7 +2403,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W70"/>
+  <dimension ref="A1:W71"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -7377,12 +7397,83 @@
         <v>2026-07-06</v>
       </c>
       <c r="W70" s="2" t="str">
-        <v>Successfully resolved the dashboard hero section layout rendering bug by completely overriding the .card background shorthand and disabling backdrop-filters on .dashboard-hero.</v>
+        <v>Successfully resolved the dashboard hero section layout rendering bug by completely overriding the .card background shorthand and disabling backdrop-filters on .dashboard-hero. Fixed C# desktop agent auto-start boot network drop resilience to suppress login prompts on slow startup connection.</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="str">
+        <v>2026-07-06</v>
+      </c>
+      <c r="B71" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C71" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D71" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E71" s="2" t="str">
+        <v>Desktop Client App</v>
+      </c>
+      <c r="F71" s="2" t="str">
+        <v>Desktop Client</v>
+      </c>
+      <c r="G71" s="2" t="str">
+        <v>Auto-Start &amp; Network Resilience</v>
+      </c>
+      <c r="H71" s="2" t="str">
+        <v>TSK-ATT-032</v>
+      </c>
+      <c r="I71" s="2" t="str">
+        <v>Implement resilient silent re-authentication on system startup</v>
+      </c>
+      <c r="J71" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K71" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L71" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M71" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N71" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O71" s="2" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="P71" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q71" s="2">
+        <v>1</v>
+      </c>
+      <c r="R71" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S71" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T71" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U71" s="2" t="str">
+        <v>2026-07-06</v>
+      </c>
+      <c r="V71" s="2" t="str">
+        <v>2026-07-06</v>
+      </c>
+      <c r="W71" s="2" t="str">
+        <v>Successfully resolved the dashboard hero section layout rendering bug by completely overriding the .card background shorthand and disabling backdrop-filters on .dashboard-hero. Fixed C# desktop agent auto-start boot network drop resilience to suppress login prompts on slow startup connection.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W71"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>